<commit_message>
adding logical response code lists to vessel electronics
</commit_message>
<xml_diff>
--- a/form_collection_templates/ros/Collection-Form-ROS-PS.xlsx
+++ b/form_collection_templates/ros/Collection-Form-ROS-PS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_collection_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CEA0C0C-E84E-AE4D-8D0C-BA5E5B8750B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCDA2B2C-C190-3247-95D7-960B6BA25FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="14800" windowHeight="16680" tabRatio="872" firstSheet="2" activeTab="7" xr2:uid="{2052CEAD-15F2-4D91-9D69-B595B4741E8A}"/>
+    <workbookView xWindow="15520" yWindow="740" windowWidth="13840" windowHeight="16680" tabRatio="872" activeTab="1" xr2:uid="{2052CEAD-15F2-4D91-9D69-B595B4741E8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="93" r:id="rId1"/>
@@ -2328,7 +2328,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="558">
+  <cellXfs count="559">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
@@ -4163,6 +4163,7 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -8959,34 +8960,34 @@
     <row r="100" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A100" s="22"/>
       <c r="B100" s="2"/>
-      <c r="C100" s="16" t="s">
+      <c r="C100" s="508" t="s">
         <v>121</v>
       </c>
       <c r="D100" s="3"/>
-      <c r="E100" s="16" t="s">
+      <c r="E100" s="508" t="s">
         <v>122</v>
       </c>
       <c r="F100" s="3"/>
       <c r="G100" s="3"/>
-      <c r="H100" s="18" t="s">
+      <c r="H100" s="558" t="s">
         <v>188</v>
       </c>
       <c r="I100" s="3"/>
-      <c r="J100" s="18" t="s">
+      <c r="J100" s="558" t="s">
         <v>123</v>
       </c>
       <c r="K100" s="3"/>
       <c r="L100" s="3"/>
       <c r="M100" s="3"/>
-      <c r="N100" s="18" t="s">
+      <c r="N100" s="558" t="s">
         <v>124</v>
       </c>
       <c r="O100" s="3"/>
-      <c r="P100" s="16" t="s">
+      <c r="P100" s="508" t="s">
         <v>125</v>
       </c>
       <c r="Q100" s="3"/>
-      <c r="S100" s="16" t="s">
+      <c r="S100" s="508" t="s">
         <v>83</v>
       </c>
       <c r="T100" s="3"/>
@@ -9062,30 +9063,30 @@
     <row r="103" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A103" s="22"/>
       <c r="B103" s="2"/>
-      <c r="C103" s="16" t="s">
+      <c r="C103" s="508" t="s">
         <v>126</v>
       </c>
       <c r="D103" s="3"/>
-      <c r="E103" s="16" t="s">
+      <c r="E103" s="508" t="s">
         <v>127</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
-      <c r="H103" s="16" t="s">
+      <c r="H103" s="508" t="s">
         <v>128</v>
       </c>
       <c r="I103" s="3"/>
-      <c r="J103" s="16" t="s">
+      <c r="J103" s="508" t="s">
         <v>129</v>
       </c>
       <c r="K103" s="3"/>
       <c r="L103" s="3"/>
       <c r="M103" s="3"/>
-      <c r="N103" s="16" t="s">
+      <c r="N103" s="508" t="s">
         <v>189</v>
       </c>
       <c r="O103" s="3"/>
-      <c r="P103" s="16" t="s">
+      <c r="P103" s="508" t="s">
         <v>130</v>
       </c>
       <c r="Q103" s="3"/>
@@ -10693,7 +10694,7 @@
       <c r="W164" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="TC3eq69EamokdKSZiO9SShM6zuYlpjJEBoJV9Ty65YKmcTF2KCBj/+gaCMC01iZ420qFTv+Q4lDawuWN4IjhMQ==" saltValue="u9007/gn6GRf2jNt2W6/FA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection selectLockedCells="1"/>
   <mergeCells count="155">
     <mergeCell ref="D113:F113"/>
     <mergeCell ref="C84:E84"/>
@@ -10874,10 +10875,23 @@
     <hyperlink ref="C94" r:id="rId19" location="fishStorageTypes" xr:uid="{C080DDC3-D9D8-3D4B-B75E-8584101CB859}"/>
     <hyperlink ref="C108:F108" r:id="rId20" location="wasteManagementCategories" display="Waste category" xr:uid="{53ECE92C-986A-6344-8281-8EE9B5454952}"/>
     <hyperlink ref="H108:Q108" r:id="rId21" location="wasteDisposalMethods" display="Storage / disposal method" xr:uid="{E49CFFDF-60AC-FE43-9AFA-94BEB08F94E0}"/>
+    <hyperlink ref="C100" r:id="rId22" location="logicalResponses" xr:uid="{C374B1BD-C21B-AF4E-ABB9-AAB70FAB1BBA}"/>
+    <hyperlink ref="E100" r:id="rId23" location="logicalResponses" xr:uid="{D003FDAD-F335-AB41-BA1F-FC289A01E96D}"/>
+    <hyperlink ref="H100" r:id="rId24" location="logicalResponses" xr:uid="{546E280B-3F1E-D146-96D7-E2954058F994}"/>
+    <hyperlink ref="J100" r:id="rId25" location="logicalResponses" xr:uid="{EF1829F6-99BC-DD46-95C2-54DC020621F7}"/>
+    <hyperlink ref="N100" r:id="rId26" location="logicalResponses" xr:uid="{B3B5D2D5-53C3-944A-8F02-ECFF79DAB1D5}"/>
+    <hyperlink ref="P100" r:id="rId27" location="logicalResponses" xr:uid="{4D4AFBEB-7DE9-A943-B362-ECCDBB57B638}"/>
+    <hyperlink ref="S100" r:id="rId28" location="logicalResponses" xr:uid="{523B1891-C70A-6F4F-8792-312C076E96DC}"/>
+    <hyperlink ref="C103" r:id="rId29" location="logicalResponses" xr:uid="{55BBEA9A-F247-E548-91BE-8E85E1B91A97}"/>
+    <hyperlink ref="E103" r:id="rId30" location="logicalResponses" xr:uid="{0E19ABAC-AB69-894C-ACE1-CA40EE8C0791}"/>
+    <hyperlink ref="H103" r:id="rId31" location="logicalResponses" xr:uid="{1DBFBC60-25C7-AF41-9C53-E929B2BDBCA7}"/>
+    <hyperlink ref="J103" r:id="rId32" location="logicalResponses" xr:uid="{4BF72DAE-AB11-8242-B79D-D1C5D789158D}"/>
+    <hyperlink ref="N103" r:id="rId33" location="logicalResponses" xr:uid="{C78386FD-5312-9544-B53F-28A54316F669}"/>
+    <hyperlink ref="P103" r:id="rId34" location="logicalResponses" xr:uid="{567E2F4B-92F4-A744-9905-2E2883CE0878}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId22"/>
-  <drawing r:id="rId23"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId35"/>
+  <drawing r:id="rId36"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
adding logcial response codes to gear
</commit_message>
<xml_diff>
--- a/form_collection_templates/ros/Collection-Form-ROS-PS.xlsx
+++ b/form_collection_templates/ros/Collection-Form-ROS-PS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_collection_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCDA2B2C-C190-3247-95D7-960B6BA25FB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218891C8-01B6-404F-B108-3DA7A8E44627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15520" yWindow="740" windowWidth="13840" windowHeight="16680" tabRatio="872" activeTab="1" xr2:uid="{2052CEAD-15F2-4D91-9D69-B595B4741E8A}"/>
+    <workbookView xWindow="15520" yWindow="740" windowWidth="13840" windowHeight="16680" tabRatio="872" activeTab="2" xr2:uid="{2052CEAD-15F2-4D91-9D69-B595B4741E8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="93" r:id="rId1"/>
@@ -483,7 +483,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="239">
   <si>
     <t>IOTC REGIONAL OBSERVER SCHEME
 VESSEL AND TRIP INFORMATION SHEET</t>
@@ -8999,36 +8999,22 @@
       <c r="A101" s="22"/>
       <c r="B101" s="2"/>
       <c r="C101" s="102"/>
-      <c r="D101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="D101" s="16"/>
       <c r="E101" s="102"/>
-      <c r="F101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="F101" s="16"/>
       <c r="G101" s="3"/>
       <c r="H101" s="102"/>
-      <c r="I101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="I101" s="16"/>
       <c r="J101" s="102"/>
-      <c r="K101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="K101" s="16"/>
       <c r="L101" s="16"/>
       <c r="M101" s="3"/>
       <c r="N101" s="102"/>
-      <c r="O101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="O101" s="16"/>
       <c r="P101" s="102"/>
-      <c r="Q101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q101" s="16"/>
       <c r="S101" s="102"/>
-      <c r="T101" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="T101" s="16"/>
       <c r="U101" s="105"/>
       <c r="V101" s="1"/>
       <c r="W101" s="4"/>
@@ -9100,32 +9086,20 @@
       <c r="A104" s="22"/>
       <c r="B104" s="2"/>
       <c r="C104" s="41"/>
-      <c r="D104" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="D104" s="16"/>
       <c r="E104" s="41"/>
-      <c r="F104" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="F104" s="16"/>
       <c r="G104" s="3"/>
       <c r="H104" s="41"/>
-      <c r="I104" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="I104" s="16"/>
       <c r="J104" s="41"/>
-      <c r="K104" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="K104" s="16"/>
       <c r="L104" s="16"/>
       <c r="M104" s="3"/>
       <c r="N104" s="41"/>
-      <c r="O104" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="O104" s="16"/>
       <c r="P104" s="41"/>
-      <c r="Q104" s="16" t="s">
-        <v>44</v>
-      </c>
+      <c r="Q104" s="16"/>
       <c r="S104" s="105"/>
       <c r="T104" s="1"/>
       <c r="U104" s="3"/>
@@ -10694,7 +10668,7 @@
       <c r="W164" s="3"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="OaeqvjErdfPtgHClBEKdHHRDEmHSSGsv3FjOeuwSJR98kOAxvoAes0aa6J9elnqI/Z08wloRLdyNM66x921CGQ==" saltValue="rV+OOS99dJSg+sZ6cWIhWw==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="155">
     <mergeCell ref="D113:F113"/>
     <mergeCell ref="C84:E84"/>
@@ -11115,23 +11089,19 @@
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="22"/>
       <c r="B8" s="2"/>
-      <c r="C8" s="235" t="s">
+      <c r="C8" s="507" t="s">
         <v>133</v>
       </c>
-      <c r="D8" s="235"/>
+      <c r="D8" s="507"/>
       <c r="E8" s="102"/>
-      <c r="F8" s="43" t="s">
-        <v>44</v>
-      </c>
+      <c r="F8" s="43"/>
       <c r="G8" s="16"/>
-      <c r="H8" s="235" t="s">
+      <c r="H8" s="507" t="s">
         <v>134</v>
       </c>
-      <c r="I8" s="235"/>
+      <c r="I8" s="507"/>
       <c r="J8" s="102"/>
-      <c r="K8" s="43" t="s">
-        <v>44</v>
-      </c>
+      <c r="K8" s="43"/>
       <c r="L8" s="16"/>
       <c r="M8" s="16"/>
       <c r="N8" s="16"/>
@@ -12348,7 +12318,7 @@
       <c r="C157" s="23"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="Kv2RWDH2Y+0kuLQvmKDBQtry4DOGwdPdosYYQg/6KcK8gwXCf+BwFwcJOaFSuJeKcx7y+vQbWsX9OPZJKiE9IQ==" saltValue="QNz3L+nzSvysH/yCPBV9kg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="L5zRAJr3/4ZI7yfHAKt7+QxnfQhu+A1SecQw2+USkySGlPkR0edJtDmqLeWII52y+NrUk4fRFxdp69Z5XZJxhg==" saltValue="OzflVGJ31T9aZoO135SY6Q==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <mergeCells count="21">
     <mergeCell ref="C12:K12"/>
     <mergeCell ref="N12:V12"/>
@@ -12373,9 +12343,13 @@
     <mergeCell ref="E4:F4"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="C8:D8" r:id="rId1" location="logicalResponses" display="Power block" xr:uid="{B21089D5-57FD-364E-A9DF-DD5D5137E93A}"/>
+    <hyperlink ref="H8:I8" r:id="rId2" location="logicalResponses" display=" Purse winch" xr:uid="{AC464E92-1C33-D74F-8297-06706FD244EF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
+  <drawing r:id="rId4"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update to code list
</commit_message>
<xml_diff>
--- a/form_collection_templates/ros/Collection-Form-ROS-PS.xlsx
+++ b/form_collection_templates/ros/Collection-Form-ROS-PS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/schirico/IOTC/IOTC_reference_forms/form_collection_templates/ros/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{044CFDBA-C902-8948-BFCF-71ADC896EBB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FD93E96-7741-8E43-B8D0-D32B33FBC1CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14680" yWindow="740" windowWidth="14680" windowHeight="16680" tabRatio="872" activeTab="5" xr2:uid="{2052CEAD-15F2-4D91-9D69-B595B4741E8A}"/>
+    <workbookView xWindow="14680" yWindow="740" windowWidth="14680" windowHeight="16680" tabRatio="872" firstSheet="2" activeTab="7" xr2:uid="{2052CEAD-15F2-4D91-9D69-B595B4741E8A}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="93" r:id="rId1"/>
@@ -21837,7 +21837,7 @@
       <c r="C259" s="23"/>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="Q2VRHBKKxyrUgJ6ig4n1WnkuPpAJokE3bZfnbsE3dqapr2GNHLvuTrlhaYvKjXgULnHuC5NU97ZaDhhY0+y2yA==" saltValue="Pnxg+pefRJezLN683n9Tww==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1"/>
   <dataConsolidate/>
   <mergeCells count="233">
     <mergeCell ref="F18:G18"/>

</xml_diff>